<commit_message>
EPBDS-14557 Improve validation and drop support of arrays as target type in vocabulary type e.g. Datatype Name<Type[]>
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-12774_Array_AliasDatatypes.xlsx
+++ b/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-12774_Array_AliasDatatypes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10410"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ekosolapova/work/demoEPBDS-12748/openl-demo/user-workspace2/DEFAULT/aliasArray/"/>
     </mc:Choice>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="26">
   <si>
     <t>Datatype Countries &lt;String[]&gt;</t>
   </si>
@@ -92,16 +92,38 @@
   </si>
   <si>
     <t>Coutries</t>
+  </si>
+  <si>
+    <t>Datatype Countries &lt;String&gt;</t>
+  </si>
+  <si>
+    <t>BE</t>
+  </si>
+  <si>
+    <t>NY</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>PL</t>
+  </si>
+  <si>
+    <t>Countries[]</t>
+  </si>
+  <si>
+    <t>SmartLookup Double smrLookup(Countries[] ctr, Integer age)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
-      <color theme="1"/>
+      <color theme="1" rgb="000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -125,7 +147,7 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -447,24 +469,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74F54271-613D-FA47-887A-42CDCE6F7996}">
-  <dimension ref="D4:G34"/>
+  <dimension ref="B4:G40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="4" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D6" t="s">
-        <v>2</v>
-      </c>
-    </row>
+    <row r="4" spans="4:6" x14ac:dyDescent="0.2"/>
+    <row r="5" spans="4:6" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="4:6" x14ac:dyDescent="0.2"/>
+    <row r="7"/>
     <row r="9" spans="4:6" x14ac:dyDescent="0.2">
       <c r="D9" s="1" t="s">
         <v>4</v>
@@ -473,146 +484,171 @@
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D10" t="s">
-        <v>5</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="D10" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" t="s" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D11" t="s">
+      <c r="D11" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="14" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D14" t="s">
+      <c r="D14" t="s" s="0">
         <v>3</v>
       </c>
     </row>
     <row r="15" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D15" t="s">
+      <c r="D15" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="16" spans="4:6" x14ac:dyDescent="0.2">
-      <c r="D16" t="s">
-        <v>5</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="D16" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" t="s" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D19" t="s">
+      <c r="D19" t="s" s="0">
         <v>9</v>
       </c>
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D20" t="s">
+      <c r="D20" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" t="s" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="21" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D21" t="s">
+      <c r="D21" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" t="s" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="22" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D22" t="s">
+      <c r="D22" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" t="s" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D26" t="s">
+      <c r="D26" t="s" s="0">
         <v>11</v>
       </c>
     </row>
     <row r="27" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D27" t="s">
+      <c r="D27" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" t="s" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="28" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D28">
+      <c r="D28" s="0">
         <v>1</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" t="s" s="0">
         <v>2</v>
       </c>
     </row>
     <row r="31" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D31" t="s">
-        <v>14</v>
+      <c r="D31" s="0" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D32" t="s">
+      <c r="D32" t="s" s="0">
         <v>18</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" t="s" s="0">
         <v>17</v>
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D33" t="s">
+      <c r="D33" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="0">
         <v>1</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="0">
         <v>4</v>
       </c>
-      <c r="G33">
+      <c r="G33" s="0">
         <v>2</v>
       </c>
     </row>
     <row r="34" spans="4:7" x14ac:dyDescent="0.2">
-      <c r="D34" t="s">
+      <c r="D34" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="0">
         <v>3</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="0">
         <v>5</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="0">
         <v>7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="s" s="0">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="0" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>